<commit_message>
Line plot for holdout amount comparison
</commit_message>
<xml_diff>
--- a/Results Dictionaries/Regression Various Splits/Holdout Split Results.xlsx
+++ b/Results Dictionaries/Regression Various Splits/Holdout Split Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffreyvanhumbeck/Documents/GitHub/Calixarenes/Results Dictionaries/Regression Various Splits/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE3178A9-56E5-EA4B-82B4-BA6AAC37748F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD56E6F-4E4F-524B-8A71-691242EFD6F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27420" yWindow="1680" windowWidth="11560" windowHeight="19660" xr2:uid="{8665AB9F-232D-F244-B7EB-71F696146AEC}"/>
+    <workbookView xWindow="22860" yWindow="7280" windowWidth="12040" windowHeight="10640" xr2:uid="{8665AB9F-232D-F244-B7EB-71F696146AEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="12">
   <si>
     <t>Net Type</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>GCN</t>
+  </si>
+  <si>
+    <t>AFP</t>
   </si>
 </sst>
 </file>
@@ -495,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5476AE7E-6A59-874D-8E2B-DFAD769237B5}">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.83203125" customWidth="1"/>
@@ -857,10 +860,10 @@
         <v>6</v>
       </c>
       <c r="D26" s="9">
-        <v>0.36</v>
+        <v>0.68</v>
       </c>
       <c r="E26" s="9">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -870,10 +873,10 @@
         <v>7</v>
       </c>
       <c r="D27" s="9">
-        <v>0.32</v>
+        <v>0.4</v>
       </c>
       <c r="E27" s="9">
-        <v>0.82</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -885,10 +888,10 @@
         <v>6</v>
       </c>
       <c r="D28" s="9">
-        <v>0.25</v>
+        <v>0.36</v>
       </c>
       <c r="E28" s="9">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -898,10 +901,10 @@
         <v>7</v>
       </c>
       <c r="D29" s="9">
-        <v>0.15</v>
+        <v>0.41</v>
       </c>
       <c r="E29" s="9">
-        <v>0.81</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -913,10 +916,10 @@
         <v>6</v>
       </c>
       <c r="D30" s="9">
-        <v>0.19</v>
+        <v>0.37</v>
       </c>
       <c r="E30" s="9">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -926,10 +929,10 @@
         <v>7</v>
       </c>
       <c r="D31" s="9">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="E31" s="9">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -941,10 +944,10 @@
         <v>6</v>
       </c>
       <c r="D32" s="9">
-        <v>0.13</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="E32" s="9">
-        <v>0.87</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -960,6 +963,120 @@
         <v>0.86</v>
       </c>
     </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B34" s="8">
+        <v>0.04</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D34" s="9">
+        <v>0.77</v>
+      </c>
+      <c r="E34" s="9">
+        <v>0.94</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="10"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35" s="9">
+        <v>0.37</v>
+      </c>
+      <c r="E35" s="9">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="10"/>
+      <c r="B36" s="8">
+        <v>0.25</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36" s="9">
+        <v>0.44</v>
+      </c>
+      <c r="E36" s="9">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="10"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="9">
+        <v>0.25</v>
+      </c>
+      <c r="E37" s="9">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="10"/>
+      <c r="B38" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38" s="9">
+        <v>0.45</v>
+      </c>
+      <c r="E38" s="9">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="10"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" s="9">
+        <v>0.43</v>
+      </c>
+      <c r="E39" s="9">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="11"/>
+      <c r="B40" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D40" s="9">
+        <v>0.22</v>
+      </c>
+      <c r="E40" s="9">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" s="12"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="13">
+        <v>0.01</v>
+      </c>
+      <c r="E41" s="13">
+        <v>0.83</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated plots with line for holdout split added
</commit_message>
<xml_diff>
--- a/Results Dictionaries/Regression Various Splits/Holdout Split Results.xlsx
+++ b/Results Dictionaries/Regression Various Splits/Holdout Split Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffreyvanhumbeck/Documents/GitHub/Calixarenes/Results Dictionaries/Regression Various Splits/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD56E6F-4E4F-524B-8A71-691242EFD6F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6723C148-B6B3-6642-AC4E-01EE6333F2C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22860" yWindow="7280" windowWidth="12040" windowHeight="10640" xr2:uid="{8665AB9F-232D-F244-B7EB-71F696146AEC}"/>
+    <workbookView xWindow="41940" yWindow="5280" windowWidth="12040" windowHeight="10640" xr2:uid="{8665AB9F-232D-F244-B7EB-71F696146AEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>